<commit_message>
Complete evidence-grounded minwon harness
</commit_message>
<xml_diff>
--- a/data/minwon_sample.xlsx
+++ b/data/minwon_sample.xlsx
@@ -360,7 +360,7 @@
     <t>교육출장여비 관련</t>
   </si>
   <si>
-    <t xml:space="preserve">안녕하세요, 울산지방해양수산청에서 지출담당을 맡고 있는 권진성이라고 합니다.
+    <t xml:space="preserve">안녕하세요, A기관에서 지출담당을 맡고 있는 담당자이라고 합니다.
 [교육훈련여비지급기준]에서 '합숙또는기숙사이용이가능한경우'에서 식비는 '당해 교육훈련기관이 청구하는 금액 또는 구내식당 가격'에 대해서 문의드리고자 합니다.
 예를 들어, 2박 3일 교육인데 '합숙또는기숙사이용이가능한경우'이지만, 비합숙으로 교육을 신청하였습니다.
 합숙또는기숙사이용을 하였다면 식비영수증을 35,000원(7식)으로 받을수있으나,
@@ -369,7 +369,7 @@
 1. 영수증(3식) + 식비규정(6식)
 2. 영수증(3식) + 식비규정(2식, 식사가 제공되지 않는 첫날 아침, 마지막날 저녁)
 어떻게 지급하는게 맞는걸까요?
-이해가 안되는 부분이 있다면 052-228-5542 or 010-9554-**** 로 연락주세요
+이해가 안되는 부분이 있다면 [연락처 생략] 로 연락주세요
 </t>
   </si>
   <si>
@@ -939,7 +939,7 @@
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" customWidth="1"/>
+    <col min="2" max="2" width="[PHONE]" customWidth="1"/>
     <col min="3" max="26" width="7.5703125" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>